<commit_message>
changed city names in xlsx "klanten" to capital letters
</commit_message>
<xml_diff>
--- a/PowerBI_Fundamentals_NL/Klanten.xlsx
+++ b/PowerBI_Fundamentals_NL/Klanten.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://quanthicsbv-my.sharepoint.com/personal/thomas_janssen_quanthics_com/Documents/00. QUANTHICS BV/02. Trainingen/00. Training Templates/PowerBI Training/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="11_F25DC773A252ABDACC10482D81D843505ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E34C8968-9A46-4039-9197-8059A2FE1367}"/>
+  <xr:revisionPtr revIDLastSave="71" documentId="11_F25DC773A252ABDACC10482D81D843505ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4D7E014-2D45-439C-A1AC-3E9A05623767}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,9 +20,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -87,27 +84,12 @@
     <t>Marieke Bos</t>
   </si>
   <si>
-    <t>Utrecht, Nederland</t>
-  </si>
-  <si>
-    <t>Amsterdam, Nederland</t>
-  </si>
-  <si>
-    <t>Maastricht, Nederland</t>
-  </si>
-  <si>
     <t>Thomas Müller</t>
   </si>
   <si>
     <t>Sabine Hoffmann</t>
   </si>
   <si>
-    <t>Munchen, Duitsland</t>
-  </si>
-  <si>
-    <t>Stuttgard, Duitsland</t>
-  </si>
-  <si>
     <t>Koen Verstraete</t>
   </si>
   <si>
@@ -117,16 +99,31 @@
     <t>Bram Van Acker</t>
   </si>
   <si>
-    <t>Gent, Belgie</t>
-  </si>
-  <si>
-    <t>Brussel, Belgie</t>
-  </si>
-  <si>
-    <t>Antwerpen, Belgie</t>
-  </si>
-  <si>
-    <t>Eindhoven, Nederland</t>
+    <t>UTRECHT, Nederland</t>
+  </si>
+  <si>
+    <t>AMSTERDAM, Nederland</t>
+  </si>
+  <si>
+    <t>MAASTRICHT, Nederland</t>
+  </si>
+  <si>
+    <t>MUNCHEN, Duitsland</t>
+  </si>
+  <si>
+    <t>STUTTGARD, Duitsland</t>
+  </si>
+  <si>
+    <t>GENT, Belgie</t>
+  </si>
+  <si>
+    <t>BRUSSEL, Belgie</t>
+  </si>
+  <si>
+    <t>ANTWERPEN, Belgie</t>
+  </si>
+  <si>
+    <t>EINDHOVEN, Nederland</t>
   </si>
 </sst>
 </file>
@@ -175,7 +172,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -487,7 +484,7 @@
         <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -501,7 +498,7 @@
         <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -515,7 +512,7 @@
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -526,10 +523,10 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -540,10 +537,10 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -554,7 +551,7 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
         <v>29</v>
@@ -568,7 +565,7 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D8" t="s">
         <v>30</v>
@@ -582,7 +579,7 @@
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D9" t="s">
         <v>31</v>
@@ -613,7 +610,7 @@
         <v>18</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>